<commit_message>
thermal optical VI and test folder update
</commit_message>
<xml_diff>
--- a/tests/test_01/build_files/Test_1_layout.xlsx
+++ b/tests/test_01/build_files/Test_1_layout.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://emailsc-my.sharepoint.com/personal/killedar_email_sc_edu/Documents/Documents/GitHub/Dataset-LPBF-Thin-Wall-and-Cube-Thermal-Optical-Monitoring/build_files/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\Dataset-LPBF-Thin-Wall-and-Cube-Thermal-Optical-Monitoring\tests\test_01\build_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="70" documentId="11_F25DC773A252ABDACC104816C91C694E5ADE58F1" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{11FC2F51-C362-4E05-AF0E-72237324C774}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{75742ADE-D947-433E-BE36-613D6A872DE0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="57480" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,13 +27,13 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="3">
   <si>
-    <t>position</t>
-  </si>
-  <si>
     <t>wall thinkness (mm)</t>
   </si>
   <si>
     <t>Cube width (mm)</t>
+  </si>
+  <si>
+    <t>position (1 -starting at left)</t>
   </si>
 </sst>
 </file>
@@ -641,22 +641,24 @@
   <dimension ref="A1:E28"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="23.44140625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="18.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23.21875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="16.109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="D1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" t="s">
         <v>1</v>
-      </c>
-      <c r="D1" t="s">
-        <v>0</v>
-      </c>
-      <c r="E1" t="s">
-        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">

</xml_diff>